<commit_message>
add some non funcional reqs
</commit_message>
<xml_diff>
--- a/Documents/Requirement_Specification.xlsx
+++ b/Documents/Requirement_Specification.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed6fcd04221c3a95/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed6fcd04221c3a95/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="358" documentId="8_{62029D73-E54E-428C-832E-C97D498E37F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCB0EFBF-98D1-4555-9DED-72CFA075E3C0}"/>
+  <xr:revisionPtr revIDLastSave="379" documentId="8_{62029D73-E54E-428C-832E-C97D498E37F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F417B3B-2822-47D6-A385-14E60BBB9FBD}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="102">
   <si>
     <r>
       <t xml:space="preserve">Moves along a </t>
@@ -139,9 +139,6 @@
     <t>Descriptions</t>
   </si>
   <si>
-    <t>Test Cases</t>
-  </si>
-  <si>
     <t>Requirement No</t>
   </si>
   <si>
@@ -262,9 +259,6 @@
     <t>R3.4</t>
   </si>
   <si>
-    <t>Return the distance to the nearest object on the right-hand side</t>
-  </si>
-  <si>
     <t>Query them at least 5 times.</t>
   </si>
   <si>
@@ -352,9 +346,6 @@
     <t>Detect free space -&gt; Park</t>
   </si>
   <si>
-    <t>No available space -&gt; Move Forward -&gt; No available space till end of the strech</t>
-  </si>
-  <si>
     <t>Car is UnParked -&gt; Unparked</t>
   </si>
   <si>
@@ -404,6 +395,27 @@
   </si>
   <si>
     <t>MoveForward(), MoveBackward(), WhereIs()</t>
+  </si>
+  <si>
+    <t>No available space -&gt; Move Forward -&gt; No available space till end of the stretch</t>
+  </si>
+  <si>
+    <t>R4.5</t>
+  </si>
+  <si>
+    <t>Noise deviation = 80 cm</t>
+  </si>
+  <si>
+    <t>R1.3</t>
+  </si>
+  <si>
+    <t>Test Cases (Ex: TC1, TC2)</t>
+  </si>
+  <si>
+    <t>Free parking distance valid detected by sensors &gt;= 150 cm</t>
+  </si>
+  <si>
+    <t>Return the distance to the nearest object on the right-hand side (mininum of the two sensors)</t>
   </si>
 </sst>
 </file>
@@ -535,25 +547,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -581,11 +575,29 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -597,13 +609,6 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -992,10 +997,10 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="20">
+      <c r="A8" s="14">
         <v>7</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="14" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1014,588 +1019,620 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A83168E-7A47-49AC-91ED-2ADE1EA7B12C}">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" style="15" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" style="9" customWidth="1"/>
     <col min="2" max="2" width="31" style="4" customWidth="1"/>
     <col min="3" max="3" width="17.44140625" customWidth="1"/>
     <col min="4" max="4" width="36.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.88671875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="17.21875" customWidth="1"/>
+    <col min="5" max="5" width="46.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>8</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>9</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>40</v>
-      </c>
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>12</v>
-      </c>
+      <c r="A4" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="20"/>
       <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="19"/>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="19"/>
+      <c r="C9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="C11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="18" t="s">
+      <c r="E11" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="18" t="s">
+      <c r="B12" s="16"/>
+      <c r="C12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
+      <c r="B14" s="16"/>
+      <c r="C14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>93</v>
-      </c>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" s="7"/>
+    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" s="17"/>
       <c r="C15" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>94</v>
+        <v>19</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>97</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="20"/>
+      <c r="C18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="1" t="s">
+      <c r="B19" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="20"/>
+      <c r="C26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B29" s="17"/>
+      <c r="C29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B31" s="20"/>
+      <c r="C31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="17"/>
+      <c r="C33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="1" t="s">
+      <c r="D34" s="1"/>
+      <c r="E34" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E26" s="18" t="s">
-        <v>95</v>
-      </c>
-      <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E28" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E30" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B31" s="10"/>
-      <c r="C31" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E31" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="8" t="s">
+      <c r="D35" s="1"/>
+      <c r="E35" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D32" s="1"/>
-      <c r="E32" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D33" s="1"/>
-      <c r="E33" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="F33" s="1"/>
+      <c r="F35" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B19:B22"/>
+    <mergeCell ref="B23:B26"/>
+    <mergeCell ref="B27:B29"/>
     <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B32:B33"/>
   </mergeCells>
-  <conditionalFormatting sqref="C2:C33">
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Functional">
-      <formula>NOT(ISERROR(SEARCH("Functional",C2)))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="C2:C35">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Non-functional">
       <formula>NOT(ISERROR(SEARCH("Non-functional",C2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Functional">
+      <formula>NOT(ISERROR(SEARCH("Functional",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1606,7 +1643,7 @@
           <x14:formula1>
             <xm:f>Stuff!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C33</xm:sqref>
+          <xm:sqref>C2:C35</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1624,17 +1661,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add a requirement for deviation sensor data
</commit_message>
<xml_diff>
--- a/Documents/Requirement_Specification.xlsx
+++ b/Documents/Requirement_Specification.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed6fcd04221c3a95/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed6fcd04221c3a95/Desktop/Halmstad_2026/Programme/Materials/Semester_1/Network_Testing_For_Embedded_Systems_DT8076/Software_Testing/Project/JUnit/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="379" documentId="8_{62029D73-E54E-428C-832E-C97D498E37F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F417B3B-2822-47D6-A385-14E60BBB9FBD}"/>
+  <xr:revisionPtr revIDLastSave="397" documentId="8_{62029D73-E54E-428C-832E-C97D498E37F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E065927-519F-4FBE-966A-292A54D86703}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="104">
   <si>
     <r>
       <t xml:space="preserve">Moves along a </t>
@@ -403,9 +403,6 @@
     <t>R4.5</t>
   </si>
   <si>
-    <t>Noise deviation = 80 cm</t>
-  </si>
-  <si>
     <t>R1.3</t>
   </si>
   <si>
@@ -416,6 +413,15 @@
   </si>
   <si>
     <t>Return the distance to the nearest object on the right-hand side (mininum of the two sensors)</t>
+  </si>
+  <si>
+    <t>R4.6</t>
+  </si>
+  <si>
+    <t>Filter value deviation &lt;= 80 cm, sensor data is valid</t>
+  </si>
+  <si>
+    <t>Filter value deviation &gt; 80 cm, sensor data is invalid</t>
   </si>
 </sst>
 </file>
@@ -575,15 +581,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -591,6 +588,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -623,6 +629,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1019,7 +1029,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A83168E-7A47-49AC-91ED-2ADE1EA7B12C}">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" style="9" customWidth="1"/>
@@ -1047,14 +1057,14 @@
         <v>8</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="15" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -1072,7 +1082,7 @@
       <c r="A3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="19"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1086,9 +1096,9 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="B4" s="20"/>
+        <v>97</v>
+      </c>
+      <c r="B4" s="17"/>
       <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1096,7 +1106,7 @@
         <v>85</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F4" s="1"/>
     </row>
@@ -1104,7 +1114,7 @@
       <c r="A5" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1122,7 +1132,7 @@
       <c r="A6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="17"/>
+      <c r="B6" s="19"/>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1138,7 +1148,7 @@
       <c r="A7" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="15" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1156,7 +1166,7 @@
       <c r="A8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="19"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1172,7 +1182,7 @@
       <c r="A9" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="19"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1188,7 +1198,7 @@
       <c r="A10" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="20"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
@@ -1196,7 +1206,7 @@
         <v>19</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F10" s="1"/>
     </row>
@@ -1204,7 +1214,7 @@
       <c r="A11" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="18" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1222,7 +1232,7 @@
       <c r="A12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="16"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
@@ -1238,7 +1248,7 @@
       <c r="A13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
@@ -1254,7 +1264,7 @@
       <c r="A14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="1" t="s">
         <v>15</v>
       </c>
@@ -1270,7 +1280,7 @@
       <c r="A15" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B15" s="17"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1278,33 +1288,33 @@
         <v>19</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>21</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="B16" s="19"/>
       <c r="C16" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="19"/>
+        <v>57</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>21</v>
+      </c>
       <c r="C17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1312,15 +1322,15 @@
         <v>85</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B18" s="20"/>
+        <v>58</v>
+      </c>
+      <c r="B18" s="16"/>
       <c r="C18" s="1" t="s">
         <v>15</v>
       </c>
@@ -1328,33 +1338,33 @@
         <v>85</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>22</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="B19" s="17"/>
       <c r="C19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="16"/>
+        <v>61</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>22</v>
+      </c>
       <c r="C20" s="1" t="s">
         <v>15</v>
       </c>
@@ -1362,15 +1372,15 @@
         <v>23</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B21" s="16"/>
+        <v>62</v>
+      </c>
+      <c r="B21" s="20"/>
       <c r="C21" s="1" t="s">
         <v>15</v>
       </c>
@@ -1378,15 +1388,15 @@
         <v>23</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F21" s="1"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B22" s="17"/>
+        <v>63</v>
+      </c>
+      <c r="B22" s="20"/>
       <c r="C22" s="1" t="s">
         <v>15</v>
       </c>
@@ -1394,33 +1404,33 @@
         <v>23</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>24</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="B23" s="19"/>
       <c r="C23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B24" s="19"/>
+        <v>66</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>24</v>
+      </c>
       <c r="C24" s="1" t="s">
         <v>15</v>
       </c>
@@ -1428,15 +1438,15 @@
         <v>25</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B25" s="19"/>
+        <v>67</v>
+      </c>
+      <c r="B25" s="16"/>
       <c r="C25" s="1" t="s">
         <v>15</v>
       </c>
@@ -1444,15 +1454,15 @@
         <v>25</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B26" s="20"/>
+        <v>68</v>
+      </c>
+      <c r="B26" s="16"/>
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
@@ -1460,33 +1470,33 @@
         <v>25</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F26" s="1"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B28" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E27" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="B28" s="16"/>
       <c r="C28" s="1" t="s">
         <v>15</v>
       </c>
@@ -1494,15 +1504,15 @@
         <v>27</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B29" s="17"/>
+        <v>75</v>
+      </c>
+      <c r="B29" s="20"/>
       <c r="C29" s="1" t="s">
         <v>15</v>
       </c>
@@ -1510,33 +1520,33 @@
         <v>27</v>
       </c>
       <c r="E29" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" s="19"/>
+      <c r="C30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E30" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="B30" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>79</v>
       </c>
       <c r="F30" s="1"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B31" s="20"/>
+        <v>80</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>28</v>
+      </c>
       <c r="C31" s="1" t="s">
         <v>15</v>
       </c>
@@ -1544,33 +1554,33 @@
         <v>29</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B32" s="15" t="s">
-        <v>31</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="B32" s="17"/>
       <c r="C32" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E32" s="12" t="s">
-        <v>93</v>
+        <v>29</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>78</v>
       </c>
       <c r="F32" s="1"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B33" s="17"/>
+        <v>82</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>31</v>
+      </c>
       <c r="C33" s="1" t="s">
         <v>15</v>
       </c>
@@ -1578,32 +1588,32 @@
         <v>30</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>33</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="B34" s="19"/>
       <c r="C34" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D34" s="1"/>
-      <c r="E34" s="11" t="s">
-        <v>34</v>
+        <v>15</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>84</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>36</v>
+        <v>32</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>16</v>
@@ -1614,20 +1624,36 @@
       </c>
       <c r="F35" s="1"/>
     </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="1"/>
+      <c r="E36" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F36" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B33:B34"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="B23:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B11:B16"/>
+    <mergeCell ref="B17:B19"/>
   </mergeCells>
-  <conditionalFormatting sqref="C2:C35">
+  <conditionalFormatting sqref="C2:C36">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Non-functional">
       <formula>NOT(ISERROR(SEARCH("Non-functional",C2)))</formula>
     </cfRule>
@@ -1643,7 +1669,7 @@
           <x14:formula1>
             <xm:f>Stuff!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C35</xm:sqref>
+          <xm:sqref>C2:C36</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Fix deviation method for sensor data, update Test Specs for IsEmpty()
</commit_message>
<xml_diff>
--- a/Documents/Requirement_Specification.xlsx
+++ b/Documents/Requirement_Specification.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed6fcd04221c3a95/Desktop/Halmstad_2026/Programme/Materials/Semester_1/Network_Testing_For_Embedded_Systems_DT8076/Software_Testing/Project/JUnit/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="397" documentId="8_{62029D73-E54E-428C-832E-C97D498E37F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E065927-519F-4FBE-966A-292A54D86703}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="8_{62029D73-E54E-428C-832E-C97D498E37F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97A67779-AA52-41DC-9FEB-74C009AA32FD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
   </bookViews>
@@ -581,6 +581,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -588,15 +597,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1064,7 +1064,7 @@
       <c r="A2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -1082,7 +1082,7 @@
       <c r="A3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1098,7 +1098,7 @@
       <c r="A4" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="17"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1114,7 +1114,7 @@
       <c r="A5" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="15" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1132,7 +1132,7 @@
       <c r="A6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="19"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1148,7 +1148,7 @@
       <c r="A7" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="18" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1166,7 +1166,7 @@
       <c r="A8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="16"/>
+      <c r="B8" s="19"/>
       <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1182,7 +1182,7 @@
       <c r="A9" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="16"/>
+      <c r="B9" s="19"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1198,7 +1198,7 @@
       <c r="A10" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="17"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
@@ -1214,7 +1214,7 @@
       <c r="A11" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="15" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1232,7 +1232,7 @@
       <c r="A12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="20"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
@@ -1248,7 +1248,7 @@
       <c r="A13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="20"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
@@ -1264,7 +1264,7 @@
       <c r="A14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="20"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="1" t="s">
         <v>15</v>
       </c>
@@ -1280,7 +1280,7 @@
       <c r="A15" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B15" s="20"/>
+      <c r="B15" s="16"/>
       <c r="C15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1296,7 +1296,7 @@
       <c r="A16" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B16" s="19"/>
+      <c r="B16" s="17"/>
       <c r="C16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1312,7 +1312,7 @@
       <c r="A17" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="18" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -1330,7 +1330,7 @@
       <c r="A18" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="16"/>
+      <c r="B18" s="19"/>
       <c r="C18" s="1" t="s">
         <v>15</v>
       </c>
@@ -1346,7 +1346,7 @@
       <c r="A19" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="17"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="1" t="s">
         <v>15</v>
       </c>
@@ -1362,7 +1362,7 @@
       <c r="A20" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1380,7 +1380,7 @@
       <c r="A21" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="20"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="1" t="s">
         <v>15</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="A22" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="20"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="1" t="s">
         <v>15</v>
       </c>
@@ -1412,7 +1412,7 @@
       <c r="A23" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="19"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="1" t="s">
         <v>15</v>
       </c>
@@ -1428,7 +1428,7 @@
       <c r="A24" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="18" t="s">
         <v>24</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1446,7 +1446,7 @@
       <c r="A25" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="16"/>
+      <c r="B25" s="19"/>
       <c r="C25" s="1" t="s">
         <v>15</v>
       </c>
@@ -1462,7 +1462,7 @@
       <c r="A26" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="16"/>
+      <c r="B26" s="19"/>
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
@@ -1478,7 +1478,7 @@
       <c r="A27" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B27" s="17"/>
+      <c r="B27" s="20"/>
       <c r="C27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1494,7 +1494,7 @@
       <c r="A28" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -1512,7 +1512,7 @@
       <c r="A29" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B29" s="20"/>
+      <c r="B29" s="16"/>
       <c r="C29" s="1" t="s">
         <v>15</v>
       </c>
@@ -1528,7 +1528,7 @@
       <c r="A30" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B30" s="19"/>
+      <c r="B30" s="17"/>
       <c r="C30" s="1" t="s">
         <v>15</v>
       </c>
@@ -1544,7 +1544,7 @@
       <c r="A31" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="18" t="s">
         <v>28</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -1562,7 +1562,7 @@
       <c r="A32" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B32" s="17"/>
+      <c r="B32" s="20"/>
       <c r="C32" s="1" t="s">
         <v>15</v>
       </c>
@@ -1578,7 +1578,7 @@
       <c r="A33" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -1596,7 +1596,7 @@
       <c r="A34" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B34" s="19"/>
+      <c r="B34" s="17"/>
       <c r="C34" s="1" t="s">
         <v>15</v>
       </c>
@@ -1642,16 +1642,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="B11:B16"/>
+    <mergeCell ref="B17:B19"/>
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="B24:B27"/>
     <mergeCell ref="B28:B30"/>
     <mergeCell ref="B31:B32"/>
     <mergeCell ref="B33:B34"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B11:B16"/>
-    <mergeCell ref="B17:B19"/>
   </mergeCells>
   <conditionalFormatting sqref="C2:C36">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Non-functional">

</xml_diff>

<commit_message>
Update requirements for move forward and backwards
</commit_message>
<xml_diff>
--- a/Documents/Requirement_Specification.xlsx
+++ b/Documents/Requirement_Specification.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed6fcd04221c3a95/Desktop/Halmstad_2026/Programme/Materials/Semester_1/Network_Testing_For_Embedded_Systems_DT8076/Software_Testing/Project/JUnit/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/crispin/Projects/Personal/School/Autonomous_Parking_Test/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="400" documentId="8_{62029D73-E54E-428C-832E-C97D498E37F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97A67779-AA52-41DC-9FEB-74C009AA32FD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38D7A02-FC59-EE45-928B-E8806CF47183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
     <sheet name="Requirements" sheetId="2" r:id="rId2"/>
     <sheet name="Stuff" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -29,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -581,15 +580,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -597,6 +587,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -953,12 +952,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BFD0E3D-BB49-40A2-B972-E4AF16E0E27F}">
   <dimension ref="A2:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="52.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -966,7 +965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -974,7 +973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -982,7 +981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -990,7 +989,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -998,7 +997,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1006,7 +1005,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="14">
         <v>7</v>
       </c>
@@ -1014,7 +1013,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1030,17 +1029,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A83168E-7A47-49AC-91ED-2ADE1EA7B12C}">
   <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.33203125" style="9" customWidth="1"/>
     <col min="2" max="2" width="31" style="4" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" customWidth="1"/>
-    <col min="4" max="4" width="36.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.88671875" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5" customWidth="1"/>
+    <col min="4" max="4" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.83203125" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>9</v>
       </c>
@@ -1060,11 +1059,11 @@
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="15" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -1078,11 +1077,11 @@
       </c>
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="19"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1094,11 +1093,11 @@
       </c>
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="20"/>
+      <c r="B4" s="17"/>
       <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1110,11 +1109,11 @@
       </c>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1128,11 +1127,11 @@
       </c>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="17"/>
+      <c r="B6" s="19"/>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1144,11 +1143,11 @@
       </c>
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="15" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1162,11 +1161,11 @@
       </c>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="19"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1178,11 +1177,11 @@
       </c>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="19"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1194,11 +1193,11 @@
       </c>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="20"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
@@ -1210,11 +1209,11 @@
       </c>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="18" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1228,11 +1227,11 @@
       </c>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="16"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
@@ -1244,11 +1243,11 @@
       </c>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
@@ -1260,11 +1259,11 @@
       </c>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="1" t="s">
         <v>15</v>
       </c>
@@ -1276,11 +1275,11 @@
       </c>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B15" s="16"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1292,11 +1291,11 @@
       </c>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B16" s="17"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1308,61 +1307,61 @@
       </c>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="E17" s="12" t="s">
         <v>90</v>
       </c>
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="19"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>91</v>
       </c>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="20"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="E19" s="12" t="s">
         <v>56</v>
       </c>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1376,11 +1375,11 @@
       </c>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="16"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="1" t="s">
         <v>15</v>
       </c>
@@ -1392,11 +1391,11 @@
       </c>
       <c r="F21" s="1"/>
     </row>
-    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="1" t="s">
         <v>15</v>
       </c>
@@ -1408,11 +1407,11 @@
       </c>
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="17"/>
+      <c r="B23" s="19"/>
       <c r="C23" s="1" t="s">
         <v>15</v>
       </c>
@@ -1424,11 +1423,11 @@
       </c>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="15" t="s">
         <v>24</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1442,11 +1441,11 @@
       </c>
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="19"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="1" t="s">
         <v>15</v>
       </c>
@@ -1458,11 +1457,11 @@
       </c>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="19"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
@@ -1474,11 +1473,11 @@
       </c>
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B27" s="20"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1490,11 +1489,11 @@
       </c>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="18" t="s">
         <v>26</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -1508,11 +1507,11 @@
       </c>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B29" s="16"/>
+      <c r="B29" s="20"/>
       <c r="C29" s="1" t="s">
         <v>15</v>
       </c>
@@ -1524,11 +1523,11 @@
       </c>
       <c r="F29" s="1"/>
     </row>
-    <row r="30" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B30" s="17"/>
+      <c r="B30" s="19"/>
       <c r="C30" s="1" t="s">
         <v>15</v>
       </c>
@@ -1540,11 +1539,11 @@
       </c>
       <c r="F30" s="1"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="15" t="s">
         <v>28</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -1558,11 +1557,11 @@
       </c>
       <c r="F31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B32" s="20"/>
+      <c r="B32" s="17"/>
       <c r="C32" s="1" t="s">
         <v>15</v>
       </c>
@@ -1574,11 +1573,11 @@
       </c>
       <c r="F32" s="1"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="18" t="s">
         <v>31</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -1592,11 +1591,11 @@
       </c>
       <c r="F33" s="1"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B34" s="17"/>
+      <c r="B34" s="19"/>
       <c r="C34" s="1" t="s">
         <v>15</v>
       </c>
@@ -1608,7 +1607,7 @@
       </c>
       <c r="F34" s="1"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
         <v>32</v>
       </c>
@@ -1624,7 +1623,7 @@
       </c>
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="8" t="s">
         <v>35</v>
       </c>
@@ -1642,16 +1641,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B11:B16"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="B24:B27"/>
     <mergeCell ref="B28:B30"/>
     <mergeCell ref="B31:B32"/>
     <mergeCell ref="B33:B34"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="B11:B16"/>
   </mergeCells>
   <conditionalFormatting sqref="C2:C36">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Non-functional">
@@ -1680,22 +1679,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6679FE4-DA14-4326-B96B-ACDA17B52EED}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>17</v>
       </c>

</xml_diff>